<commit_message>
feat: auto-populate SOTP Cross-Check table from DCF model values
generate_sotp.py now finds the latest DCF model for the ticker,
opens it via win32com to evaluate formulas, and injects the four
fair values (PGM, Exit Multiple, EV/EBITDA, PER) into the
Cross-Check table on the Cover & Thesis sheet. Falls back
gracefully if no DCF model exists or Excel is unavailable.

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/models/6363_SOTP_Model.xlsx
+++ b/models/6363_SOTP_Model.xlsx
@@ -718,7 +718,9 @@
           <t>DCF — Perpetuity Growth</t>
         </is>
       </c>
-      <c r="C13" s="9" t="n"/>
+      <c r="C13" s="9" t="n">
+        <v>3207</v>
+      </c>
       <c r="D13" s="10">
         <f>(C13-$C$12)/$C$12</f>
         <v/>
@@ -730,7 +732,9 @@
           <t>DCF — Exit Multiple</t>
         </is>
       </c>
-      <c r="C14" s="9" t="n"/>
+      <c r="C14" s="9" t="n">
+        <v>5507</v>
+      </c>
       <c r="D14" s="10">
         <f>(C14-$C$12)/$C$12</f>
         <v/>
@@ -742,7 +746,9 @@
           <t>Comps — EV/EBITDA</t>
         </is>
       </c>
-      <c r="C15" s="9" t="n"/>
+      <c r="C15" s="9" t="n">
+        <v>2718</v>
+      </c>
       <c r="D15" s="10">
         <f>(C15-$C$12)/$C$12</f>
         <v/>
@@ -754,7 +760,9 @@
           <t>Comps — PER</t>
         </is>
       </c>
-      <c r="C16" s="9" t="n"/>
+      <c r="C16" s="9" t="n">
+        <v>2322</v>
+      </c>
       <c r="D16" s="10">
         <f>(C16-$C$12)/$C$12</f>
         <v/>

</xml_diff>